<commit_message>
ci: add unified 4-pillar enterprise CI/CD pipeline, appium mobile framework, vulnerability test suite, and load testing
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,8 +31,18 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +53,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F2937"/>
         <bgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -72,9 +88,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -442,16 +464,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -488,6 +510,154 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TC-AUTH-010</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Mobile auth validation 10: Sign-in screen escape handling</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Simulated boundary verification failure for TC-AUTH-010: Response mismatch.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>D:\Medical report analyzer\Test Results\Screenshots\FAIL_TC-AUTH-010_1793197603093.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TC-FORM-008</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Forms</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Form interaction scenario 8: Form field state validation 8</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Simulated boundary verification failure for TC-FORM-008: Response mismatch.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>D:\Medical report analyzer\Test Results\Screenshots\FAIL_TC-FORM-008_1793197603221.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TC-ERR-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Error Handling</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Error resilience scenario 3: Corrupt PDF document upload error</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Simulated boundary verification failure for TC-ERR-003: Response mismatch.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>D:\Medical report analyzer\Test Results\Screenshots\FAIL_TC-ERR-003_1793197603374.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TC-UPL-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>File Upload</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Mobile document upload scenario 4: Oversized 25MB file upload rejection</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Simulated boundary verification failure for TC-UPL-004: Response mismatch.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>D:\Medical report analyzer\Test Results\Screenshots\FAIL_TC-UPL-004_1793197603489.png</t>
         </is>
       </c>
     </row>

</xml_diff>